<commit_message>
Model no and attribute matching added
</commit_message>
<xml_diff>
--- a/data/Brands.xlsx
+++ b/data/Brands.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4A5908A-0263-4555-BF3D-F4145DE615DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{737057C5-5C17-4D1B-AD90-1F7C613450A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11,7 +11,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$A$359</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$A$358</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1007" uniqueCount="1007">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1006" uniqueCount="1006">
   <si>
     <t>Unbrako</t>
   </si>
@@ -866,9 +866,6 @@
   </si>
   <si>
     <t>Polyhydron</t>
-  </si>
-  <si>
-    <t>Rr</t>
   </si>
   <si>
     <t>Solo</t>
@@ -3368,7 +3365,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A1011"/>
+  <dimension ref="A1:A1010"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="27.36328125" bestFit="1" customWidth="1"/>
@@ -3376,7 +3373,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
@@ -5164,8 +5161,8 @@
         <v>356</v>
       </c>
     </row>
-    <row r="359" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A359" t="s">
+    <row r="360" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A360" t="s">
         <v>357</v>
       </c>
     </row>
@@ -5564,8 +5561,8 @@
         <v>436</v>
       </c>
     </row>
-    <row r="440" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A440" t="s">
+    <row r="441" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A441" t="s">
         <v>437</v>
       </c>
     </row>
@@ -5909,8 +5906,8 @@
         <v>505</v>
       </c>
     </row>
-    <row r="510" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A510" t="s">
+    <row r="511" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A511" t="s">
         <v>506</v>
       </c>
     </row>
@@ -6279,8 +6276,8 @@
         <v>579</v>
       </c>
     </row>
-    <row r="585" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A585" t="s">
+    <row r="586" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A586" t="s">
         <v>580</v>
       </c>
     </row>
@@ -8404,13 +8401,8 @@
         <v>1004</v>
       </c>
     </row>
-    <row r="1011" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A1011" t="s">
-        <v>1005</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:A359" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:A358" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>